<commit_message>
New ranking and problems
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kokimoto\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA2823B0-C478-4A0A-B73F-38CB016E37F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BC8B503-B3D9-429A-A932-A3B96B00439D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -681,15 +681,15 @@
         <v>100</v>
       </c>
       <c r="L2" s="5">
-        <v>50.4</v>
+        <v>89</v>
       </c>
       <c r="M2" s="5">
         <f>SUM(I2:L2)</f>
-        <v>350.4</v>
+        <v>389</v>
       </c>
       <c r="N2" s="6">
         <f>SUM(H2,M2)</f>
-        <v>610.41</v>
+        <v>649.01</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="15">

</xml_diff>